<commit_message>
Separação de doses + opção Digitar outra dose
</commit_message>
<xml_diff>
--- a/bmed-lme-app/data/banco_dados_lme_com_anamnese.xlsx
+++ b/bmed-lme-app/data/banco_dados_lme_com_anamnese.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>100 mg – cápsula; 200 mg – cápsula</t>
+          <t>100 mg – cápsula|200 mg – cápsula</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>125 mg, 250 mg e 500 mg – comprimido</t>
+          <t>125 mg - comprimido|250 mg - comprimido|500 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>500 mg e 1000 mg – comprimido</t>
+          <t>500 mg - comprimido|1000 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido</t>
+          <t>5 mg - comprimido|10 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>25 mg – frasco-ampola; 50 mg – seringa preenchida - Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
+          <t>25 mg – frasco-ampola|50 mg – seringa preenchida - Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>25 mg – frasco-ampola; 50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
+          <t>25 mg – frasco-ampola|50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>25 mg injetável – frasco-ampola; 50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
+          <t>25 mg injetável – frasco-ampola|50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0,5 mg; 0,75 mg; 1,0 mg – comprimido</t>
+          <t>0,5 mg|0,75 mg|1,0 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2,5 mg – ampola</t>
+          <t>2 - ampola|5 mg - ampola</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0,5 mg – cápsula</t>
+          <t>0 - cápsula|5 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0,1 mg – comprimido</t>
+          <t>0 - comprimido|1 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0,1 mg – comprimido</t>
+          <t>0 - comprimido|1 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Formoterol 12 mcg + Budesonida 400 mcg – cápsula inalante ou pó inalante; Formoterol 6 mcg + Budesonida 200 mcg – cápsula inalante</t>
+          <t>Formoterol 12 mcg + Budesonida 400 mcg – cápsula inalante ou pó inalante|Formoterol 6 mcg + Budesonida 200 mcg – cápsula inalante</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1.000 UI, 2.000 UI, 3.000 UI, 4.000 UI e 10.000 UI injetável – frasco-ampola</t>
+          <t>1.000 UI - frasco-ampola|2.000 UI - frasco-ampola|3.000 UI - frasco-ampola|4.000 UI - frasco-ampola|10.000 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Formoterol 12 mcg + Budesonida 400 mcg – cápsula inalante ou pó inalante; Formoterol 6 mcg + Budesonida 200 mcg – cápsula inalante ou pó inalante</t>
+          <t>Formoterol 12 mcg + Budesonida 400 mcg – cápsula inalante ou pó inalante|Formoterol 6 mcg + Budesonida 200 mcg – cápsula inalante ou pó inalante</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>300 mg e 400 mg – cápsula</t>
+          <t>300 mg - cápsula|400 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>300 mg e 400 mg – cápsula</t>
+          <t>300 mg - cápsula|400 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>8 mg, 16 mg e 24 mg – cápsula de liberação prolongada</t>
+          <t>8 mg - cápsula de liberação prolongada|16 mg - cápsula de liberação prolongada|24 mg - cápsula de liberação prolongada</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>600 mg e 900 mg – comprimido</t>
+          <t>600 mg - comprimido|900 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>3,6 mg e 10,8 mg injetável – seringa preenchida</t>
+          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>3,6 mg e 10,8 mg injetável – seringa preenchida</t>
+          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>3,6 mg e 10,8 mg injetável – seringa preenchida</t>
+          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1.000 UI, 2.000 UI, 3.000 UI, 4.000 UI e 10.000 UI injetável – frasco-ampola</t>
+          <t>1.000 UI - frasco-ampola|2.000 UI - frasco-ampola|3.000 UI - frasco-ampola|4.000 UI - frasco-ampola|10.000 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>100 mg – comprimido; 500 mg – cápsula</t>
+          <t>100 mg – comprimido|500 mg – cápsula</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0,5g, 1g e 5,0g injetável – frasco</t>
+          <t>0 - frasco|5g - frasco|1g - frasco|5 - frasco|0g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>10 mg e 20 mg – cápsula</t>
+          <t>10 mg - cápsula|20 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|50 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>60 mg, 90 mg e 120 mg injetável – seringa preenchida</t>
+          <t>60 mg - seringa preenchida|90 mg - seringa preenchida|120 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>3,75 mg injetável – frasco-ampola</t>
+          <t>3 - frasco-ampola|75 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>3,75 mg injetável – frasco-ampola</t>
+          <t>3 - frasco-ampola|75 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>400 mg, 500 mg, 800 mg – comprimido</t>
+          <t>400 mg - comprimido|500 mg - comprimido|800 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>400 mg, 500 mg e 800 mg – comprimido; 250 mg, 500 mg e 1000 mg – supositório; 1 g + diluente 100 mL – enema; 2 g – grânulos de liberação prolongada (por sachê)</t>
+          <t>400 mg, 500 mg e 800 mg – comprimido|250 mg, 500 mg e 1000 mg – supositório|1 g + diluente 100 mL – enema|2 g – grânulos de liberação prolongada (por sachê)</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido; 10 mg/mL injetável – ampola de 1mL</t>
+          <t>5 mg e 10 mg – comprimido|10 mg/mL injetável – ampola de 1mL</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>25mg/mL – injetável, frasco-ampola de 2mL; 2,5mg – comprimido</t>
+          <t>25mg/mL – injetável, frasco-ampola de 2mL|2,5mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4670,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>25 mg/mL – injetável, ampola de 2 mL; 2,5 mg – comprimido</t>
+          <t>25 mg/mL – injetável, ampola de 2 mL|2,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>180 mg e 360 mg – comprimido</t>
+          <t>180 mg - comprimido|360 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5006,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>180 mg e 360 mg – comprimido</t>
+          <t>180 mg - comprimido|360 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5062,7 +5062,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>180 mg e 360 mg – comprimido</t>
+          <t>180 mg - comprimido|360 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>10 mg/mL injetável – ampola de 1 mL; 10 mg/mL solução oral – frasco de 60 mL; 10 mg e 30 mg – comprimido; 30 mg, 60 mg e 100 mg – cápsula de liberação controlada.</t>
+          <t>10 mg/mL injetável – ampola de 1 mL|10 mg/mL solução oral – frasco de 60 mL|10 mg e 30 mg – comprimido|30 mg, 60 mg e 100 mg – cápsula de liberação controlada.</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>250mg e 500mg – comprimido</t>
+          <t>250mg - comprimido|500mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>250 mg e 500 mg – comprimido</t>
+          <t>250 mg - comprimido|500 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Lar 10 mg, 20 mg e 30 mg injetável – frasco-ampola; 0,1 mg/ml injetável – ampola</t>
+          <t>Lar 10 mg, 20 mg e 30 mg injetável – frasco-ampola|0,1 mg/ml injetável – ampola</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido</t>
+          <t>5 mg - comprimido|10 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido</t>
+          <t>5 mg - comprimido|10 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>10.000 UI e 25.000 UI – cápsula</t>
+          <t>10.000 UI - cápsula|25.000 UI - cápsula</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>10.000 UI e 25.000 UI de lipase – cápsula</t>
+          <t>10.000 UI - cápsula|25.000 UI de lipase - cápsula</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>0,125 mg, 0,25 mg e 1 mg – comprimido</t>
+          <t>0 - comprimido|125 mg - comprimido|0 - comprimido|25 mg - comprimido|1 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>10 mg, 20 mg e 40 mg – comprimido</t>
+          <t>10 mg - comprimido|20 mg - comprimido|40 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>100 mg e 250 mg – comprimido</t>
+          <t>100 mg - comprimido|250 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>25 mg, 100 mg, 200 mg e 300 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido|200 mg - comprimido|300 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>25 mg, 100 mg, 200 mg e 300 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido|200 mg - comprimido|300 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido revestido</t>
+          <t>5 mg - comprimido revestido|10 mg - comprimido revestido</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>1 mg, 2 mg e 3 mg – comprimido</t>
+          <t>1 mg - comprimido|2 mg - comprimido|3 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>1 mg, 2 mg e 3 mg – comprimido</t>
+          <t>1 mg - comprimido|2 mg - comprimido|3 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>1,5 mg, 3 mg, 4,5 mg e 6 mg – cápsula; 2,0 mg/ml solução oral – frasco de 120ml; 9 mg e 18 mg - adesivo transdérmico.</t>
+          <t>1,5 mg, 3 mg, 4,5 mg e 6 mg – cápsula|2,0 mg/ml solução oral – frasco de 120ml|9 mg e 18 mg - adesivo transdérmico.</t>
         </is>
       </c>
     </row>
@@ -6686,7 +6686,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>25 mg e 50 mg – comprimido</t>
+          <t>25 mg - comprimido|50 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>10 mg, 20 mg, 40 mg, 80 mg – comprimido</t>
+          <t>10 mg - comprimido|20 mg - comprimido|40 mg - comprimido|80 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6854,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>1 mg e 2 mg – drágea</t>
+          <t>1 mg - drágea|2 mg - drágea</t>
         </is>
       </c>
     </row>
@@ -6910,7 +6910,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>4 UI injetável (1,33 mg por frasco-ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
+          <t>4 UI injetável (1 - ampola), 12 UI injetável (4 mg por frasco-ampola)|33 mg por frasco - ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>4 UI injetável (1,33 mg por frasco-ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
+          <t>4 UI injetável (1 - ampola), 12 UI injetável (4 mg por frasco-ampola)|33 mg por frasco - ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
         </is>
       </c>
     </row>
@@ -7470,7 +7470,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>1 mg e 5 mg – cápsula</t>
+          <t>1 mg - cápsula|5 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>1 mg e 5 mg – cápsula</t>
+          <t>1 mg - cápsula|5 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7694,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|50 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>100 UI e 500 UI injetável – frasco-ampola</t>
+          <t>100 UI - frasco-ampola|500 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>100 UI e 500 UI injetável – frasco-ampola</t>
+          <t>100 UI - frasco-ampola|500 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -7918,7 +7918,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>40 mg e 80 mg – cápsula</t>
+          <t>40 mg - cápsula|80 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>40 mg e 80 mg – cápsula</t>
+          <t>40 mg - cápsula|80 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -8142,7 +8142,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>25 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|50 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -8254,7 +8254,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>5 mg e 10 mg – comprimido</t>
+          <t>5 mg - comprimido|10 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>25 mg, 100 mg, 200 mg, 300 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido|200 mg - comprimido|300 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -8366,7 +8366,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>1 mg, 2 mg e 3 mg – comprimido</t>
+          <t>1 mg - comprimido|2 mg - comprimido|3 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -8422,7 +8422,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>1 mg, 2 mg e 3 mg – comprimido; 1 mg/ml – solução oral (por frasco de 30 ml)</t>
+          <t>1 mg, 2 mg e 3 mg – comprimido|1 mg/ml – solução oral (por frasco de 30 ml)</t>
         </is>
       </c>
     </row>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>250 mg e 500 mg – comprimido</t>
+          <t>250 mg - comprimido|500 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -9206,7 +9206,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>0,5 mg; 0,75 mg; 1,0 mg – comprimido</t>
+          <t>0,5 mg|0,75 mg|1,0 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -9430,7 +9430,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>180 mg e 360 mg – comprimido</t>
+          <t>180 mg - comprimido|360 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -9486,7 +9486,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>1 mg e 5 mg – cápsula</t>
+          <t>1 mg - cápsula|5 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>25 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -9710,7 +9710,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>30 mg e 60 mg – comprimido</t>
+          <t>30 mg - comprimido|60 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>0,25 mcg – cápsula</t>
+          <t>0 - cápsula|25 mcg - cápsula</t>
         </is>
       </c>
     </row>
@@ -9822,7 +9822,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>0,58 mg/ml injetável - frasco com 5 mL</t>
+          <t>0 - frasco com 5 mL|58 mg/ml injetável - frasco com 5 mL</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>3,75 mg e 11,25 mg injetável – frasco-ampola</t>
+          <t>3 - frasco-ampola|75 mg - frasco-ampola|11 - frasco-ampola|25 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>3,75 mg e 11,25 mg injetável – frasco-ampola</t>
+          <t>3 - frasco-ampola|75 mg - frasco-ampola|11 - frasco-ampola|25 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>120mg e 240mg – cápsula</t>
+          <t>120mg - cápsula|240mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -10326,7 +10326,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>0,5 mg; 0,75 mg; 1,0 mg – comprimido</t>
+          <t>0,5 mg|0,75 mg|1,0 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11000,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>3.000.000 UI, 5.000.000 UI, 10.000.000 UI injetável – frasco-ampola</t>
+          <t>3.000.000 UI - frasco-ampola|5.000.000 UI - frasco-ampola|10.000.000 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -11168,7 +11168,7 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>1 mg e 2 mg – drágea</t>
+          <t>1 mg - drágea|2 mg - drágea</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11224,7 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>20mg - cápsula, 61mg - cápsulas</t>
+          <t>20mg - cápsula|61mg - cápsulas</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>250 mg, 500 mg, 750 mg, 1000 mg por comprimido, 100 mg/mL solução oral – frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL</t>
+          <t>250 mg - frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL|500 mg - frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL|750 mg - frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL|1000 mg por comprimido - frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL|100 mg/mL solução oral - frasco de 100mL e 100 mg/mL solução oral – frasco de 150mL</t>
         </is>
       </c>
     </row>
@@ -11392,7 +11392,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>62,5 mg e 125 mg – comprimido revestido</t>
+          <t>62 - comprimido revestido|5 mg - comprimido revestido|125 mg - comprimido revestido</t>
         </is>
       </c>
     </row>
@@ -11448,7 +11448,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>25 mg, 50 mg e 100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -11504,7 +11504,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>25 mg injetável – frasco ampola; 50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
+          <t>25 mg injetável – frasco ampola|50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
         </is>
       </c>
     </row>
@@ -11560,7 +11560,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>45mg/0,5ml injetável – seringa preenchida</t>
+          <t>45mg/0 - seringa preenchida|5ml injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -11672,7 +11672,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>25mg e 50mg – comprimidos revestidos</t>
+          <t>25mg - comprimidos revestidos|50mg - comprimidos revestidos</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>40 mg injetável – seringa preenchida; 40 mg injetável – frasco-ampola</t>
+          <t>40 mg injetável – seringa preenchida|40 mg injetável – frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -12288,7 +12288,7 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/ml – solução oral – frasco de 50 ml</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/ml – solução oral – frasco de 50 ml</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>25 mg – frasco-ampola; 50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
+          <t>25 mg – frasco-ampola|50 mg – seringa preenchida – Originador (Enbrel®) e Biossimilar (Brenzys®)</t>
         </is>
       </c>
     </row>
@@ -12624,7 +12624,7 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>250mg e 500mg – comprimido</t>
+          <t>250mg - comprimido|500mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -12736,7 +12736,7 @@
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>25mg/ml – injetável, frasco-ampola de 2ml; 2,5mg – comprimido</t>
+          <t>25mg/ml – injetável, frasco-ampola de 2ml|2,5mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -12848,7 +12848,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>2,5 g e 5,0 g injetável – frasco</t>
+          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -13128,7 +13128,7 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>1 mg e 2 mg – drágea</t>
+          <t>1 mg - drágea|2 mg - drágea</t>
         </is>
       </c>
     </row>
@@ -13184,7 +13184,7 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>200 mcg – cápsula inalante, 400 mcg – cápsula inalante</t>
+          <t>200 mcg – cápsula inalante|400 mcg – cápsula inalante</t>
         </is>
       </c>
     </row>
@@ -13240,7 +13240,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>1 mg – 930 cápsulas; 5 mg – 248 cápsulas</t>
+          <t>1 mg – 930 cápsulas|5 mg – 248 cápsulas</t>
         </is>
       </c>
     </row>
@@ -13296,7 +13296,7 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>0,5 mg; 0,75 mg; 1 mg – comprimido</t>
+          <t>0,5 mg|0,75 mg|1 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -13464,7 +13464,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>2,4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
+          <t>2 - frasco-ampola (5 ml)|4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
         </is>
       </c>
     </row>
@@ -13520,7 +13520,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>2,4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
+          <t>2 - frasco-ampola (5 ml)|4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
         </is>
       </c>
     </row>
@@ -13576,7 +13576,7 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>200 mcg – cápsula inalante, 400 mcg – cápsula inalante</t>
+          <t>200 mcg – cápsula inalante|400 mcg – cápsula inalante</t>
         </is>
       </c>
     </row>
@@ -13744,7 +13744,7 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>0,75 mg/mL pó para solução oral – frasco 80 mL</t>
+          <t>0 - frasco 80 mL|75 mg/mL pó para solução oral - frasco 80 mL</t>
         </is>
       </c>
     </row>
@@ -13800,7 +13800,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>0,75 mg/mL pó para solução oral – frasco 80 mL</t>
+          <t>0 - frasco 80 mL|75 mg/mL pó para solução oral - frasco 80 mL</t>
         </is>
       </c>
     </row>
@@ -13856,7 +13856,7 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>0,5 mg – comprimido</t>
+          <t>0 - comprimido|5 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -13968,7 +13968,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>0,5mg – comprimido</t>
+          <t>0 - comprimido|5mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -14024,7 +14024,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>50 mcg/g (0,005%) pomada – bisnaga de 30g</t>
+          <t>50 mcg/g (0 - bisnaga de 30g|005%) pomada - bisnaga de 30g</t>
         </is>
       </c>
     </row>
@@ -14192,7 +14192,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>0,25 mcg – cápsula</t>
+          <t>0 - cápsula|25 mcg - cápsula</t>
         </is>
       </c>
     </row>
@@ -14248,7 +14248,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>0,25 mcg – cápsula</t>
+          <t>0 - cápsula|25 mcg - cápsula</t>
         </is>
       </c>
     </row>
@@ -14304,7 +14304,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>0,25 mcg – cápsula</t>
+          <t>0 - cápsula|25 mcg - cápsula</t>
         </is>
       </c>
     </row>
@@ -14812,7 +14812,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -14924,7 +14924,7 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -14980,7 +14980,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15036,7 +15036,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/ml – solução oral – frasco de 50 ml</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/ml – solução oral – frasco de 50 ml</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>25 mg, 50 mg e 100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15148,7 +15148,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15204,7 +15204,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>25 mg, 50 mg e 100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15260,7 +15260,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg, 100 mg – cápsula</t>
+          <t>25 mg - cápsula|50 mg - cápsula|100 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -15372,7 +15372,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>10 mg, 25 mg, 50 mg e 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>10 mg, 25 mg, 50 mg e 100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15428,7 +15428,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15484,7 +15484,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15540,7 +15540,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15596,7 +15596,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>25 mg, 50 mg e 100 mg – cápsula; 100 mg/mL solução oral – frasco de 50 mL</t>
+          <t>25 mg, 50 mg e 100 mg – cápsula|100 mg/mL solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -15820,7 +15820,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>40 mg injetável – seringa preenchida; 40 mg injetável – frasco-ampola</t>
+          <t>40 mg injetável – seringa preenchida|40 mg injetável – frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -15932,7 +15932,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>10 mg e 20 mg – comprimido</t>
+          <t>10 mg - comprimido|20 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -16156,7 +16156,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>25 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -16212,7 +16212,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>25 mg e 100 mg – comprimido</t>
+          <t>25 mg - comprimido|100 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -16268,7 +16268,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>40 mg injetável – seringa preenchida; 40 mg injetável – frasco-ampola – Biossimilar (Amgevita®)</t>
+          <t>40 mg injetável – seringa preenchida|40 mg injetável – frasco-ampola – Biossimilar (Amgevita®)</t>
         </is>
       </c>
     </row>
@@ -16436,7 +16436,7 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>50 mg, 150 mg, 300 mg – comprimido</t>
+          <t>50 mg - comprimido|150 mg - comprimido|300 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -16492,7 +16492,7 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>10 mg – comprimido, 25 mg – comprimido</t>
+          <t>10 mg – comprimido|25 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -16548,7 +16548,7 @@
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>10 mg e 25 mg – cápsula</t>
+          <t>10 mg - cápsula|25 mg - cápsula</t>
         </is>
       </c>
     </row>
@@ -16604,7 +16604,7 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>1.000 UI, 2.000 UI, 3.000 UI, 4.000 UI e 10.000 UI injetável – frasco-ampola</t>
+          <t>1.000 UI - frasco-ampola|2.000 UI - frasco-ampola|3.000 UI - frasco-ampola|4.000 UI - frasco-ampola|10.000 UI injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -16772,7 +16772,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>200 mg – drágea ou comprimido; 400 mg – comprimido de desintegração lenta</t>
+          <t>200 mg – drágea ou comprimido|400 mg – comprimido de desintegração lenta</t>
         </is>
       </c>
     </row>
@@ -16884,7 +16884,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -16940,7 +16940,7 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>10 mg – cápsula; 25 mg – cápsula; 50 mg – cápsula; 100 mg – cápsula; 100 mg/mL – solução oral – frasco de 50 mL</t>
+          <t>10 mg – cápsula|25 mg – cápsula|50 mg – cápsula|100 mg – cápsula|100 mg/mL – solução oral – frasco de 50 mL</t>
         </is>
       </c>
     </row>
@@ -16996,7 +16996,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>3 mg/mL solução oral – frasco de 120mL; 30 mg/ml injetável – ampola de 2mL; 30 mg e 60 mg – comprimido</t>
+          <t>3 mg/mL solução oral – frasco de 120mL|30 mg/ml injetável – ampola de 2mL|30 mg e 60 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -17052,7 +17052,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>100 mg – cápsula; 200 mg – cápsula</t>
+          <t>100 mg – cápsula|200 mg – cápsula</t>
         </is>
       </c>
     </row>
@@ -17108,7 +17108,7 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>25 mg e 50 mg – comprimido</t>
+          <t>25 mg - comprimido|50 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -17164,7 +17164,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>40 mg/0,4 mL; 60 mg/0,6 mL – seringa preenchida</t>
+          <t>40 mg/0,4 mL|60 mg/0,6 mL – seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -17276,7 +17276,7 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>0,5; 1,0; 2,5; 5,0 g injetável – frasco</t>
+          <t>0,5|1,0|2,5|5,0 g injetável – frasco</t>
         </is>
       </c>
     </row>
@@ -17448,7 +17448,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>5,0 mcg/mL – ampola de 1 mL</t>
+          <t>5 - ampola de 1 mL|0 mcg/mL - ampola de 1 mL</t>
         </is>
       </c>
     </row>
@@ -17504,7 +17504,7 @@
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>Rituximabe 500mg injetável- frasco ampola de 50ml; Rituximabe 100mg injetável – frasco ampola de 10ml (somente para complementação da dose)</t>
+          <t>Rituximabe 500mg injetável- frasco ampola de 50ml|Rituximabe 100mg injetável – frasco ampola de 10ml (somente para complementação da dose)</t>
         </is>
       </c>
     </row>
@@ -17560,7 +17560,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>1,5 mg; 3 mg; 4,5 mg; 6 mg – cápsula; 9 mg; 18 mg – adesivo transdérmico</t>
+          <t>1,5 mg|3 mg|4,5 mg|6 mg – cápsula|9 mg|18 mg – adesivo transdérmico</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update repository with local changes
</commit_message>
<xml_diff>
--- a/bmed-lme-app/data/banco_dados_lme_com_anamnese.xlsx
+++ b/bmed-lme-app/data/banco_dados_lme_com_anamnese.xlsx
@@ -1482,7 +1482,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2 - ampola|5 mg - ampola</t>
+          <t>2,5 mg – ampola</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0 - cápsula|5 mg - cápsula</t>
+          <t>0,5 mg – cápsula</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0 - comprimido|1 mg - comprimido</t>
+          <t>0,1 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0 - comprimido|1 mg - comprimido</t>
+          <t>0,1 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
+          <t>3,6 mg - seringa preenchida|10,8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
+          <t>3,6 mg - seringa preenchida|10,8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>3 - seringa preenchida|6 mg - seringa preenchida|10 - seringa preenchida|8 mg injetável - seringa preenchida</t>
+          <t>3,6 mg - seringa preenchida|10,8 mg injetável - seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0 - frasco|5g - frasco|1g - frasco|5 - frasco|0g injetável - frasco</t>
+          <t>0,5g - frasco|1g - frasco|5,0g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>3 - frasco-ampola|75 mg injetável - frasco-ampola</t>
+          <t>3,75 mg injetável – frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>3 - frasco-ampola|75 mg injetável - frasco-ampola</t>
+          <t>3,75 mg injetável – frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>0 - comprimido|125 mg - comprimido|0 - comprimido|25 mg - comprimido|1 mg - comprimido</t>
+          <t>0,125 mg - comprimido|0,25 mg - comprimido|1 mg - comprimido</t>
         </is>
       </c>
     </row>
@@ -6910,7 +6910,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>4 UI injetável (1 - ampola), 12 UI injetável (4 mg por frasco-ampola)|33 mg por frasco - ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
+          <t>4 UI injetável (1,33 mg por frasco-ampola)|12 UI injetável (4 mg por frasco-ampola)</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>4 UI injetável (1 - ampola), 12 UI injetável (4 mg por frasco-ampola)|33 mg por frasco - ampola), 12 UI injetável (4 mg por frasco-ampola)</t>
+          <t>4 UI injetável (1,33 mg por frasco-ampola)|12 UI injetável (4 mg por frasco-ampola)</t>
         </is>
       </c>
     </row>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>0 - cápsula|25 mcg - cápsula</t>
+          <t>0,25 mcg – cápsula</t>
         </is>
       </c>
     </row>
@@ -9822,7 +9822,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>0 - frasco com 5 mL|58 mg/ml injetável - frasco com 5 mL</t>
+          <t>0,58 mg/ml injetável - frasco com 5 mL</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>3 - frasco-ampola|75 mg - frasco-ampola|11 - frasco-ampola|25 mg injetável - frasco-ampola</t>
+          <t>3,75 mg - frasco-ampola|11,25 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>3 - frasco-ampola|75 mg - frasco-ampola|11 - frasco-ampola|25 mg injetável - frasco-ampola</t>
+          <t>3,75 mg - frasco-ampola|11,25 mg injetável - frasco-ampola</t>
         </is>
       </c>
     </row>
@@ -11392,7 +11392,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>62 - comprimido revestido|5 mg - comprimido revestido|125 mg - comprimido revestido</t>
+          <t>62,5 mg - comprimido revestido|125 mg - comprimido revestido</t>
         </is>
       </c>
     </row>
@@ -11560,7 +11560,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>45mg/0 - seringa preenchida|5ml injetável - seringa preenchida</t>
+          <t>45mg/0,5ml injetável – seringa preenchida</t>
         </is>
       </c>
     </row>
@@ -12848,7 +12848,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>2 - frasco|5 g - frasco|5 - frasco|0 g injetável - frasco</t>
+          <t>2,5 g - frasco|5,0 g injetável - frasco</t>
         </is>
       </c>
     </row>
@@ -13464,7 +13464,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>2 - frasco-ampola (5 ml)|4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
+          <t>2,4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
         </is>
       </c>
     </row>
@@ -13520,7 +13520,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>2 - frasco-ampola (5 ml)|4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
+          <t>2,4 mg/ml solução injetável - frasco-ampola (5 ml)</t>
         </is>
       </c>
     </row>
@@ -13744,7 +13744,7 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>0 - frasco 80 mL|75 mg/mL pó para solução oral - frasco 80 mL</t>
+          <t>0,75 mg/mL pó para solução oral – frasco 80 mL</t>
         </is>
       </c>
     </row>
@@ -13800,7 +13800,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>0 - frasco 80 mL|75 mg/mL pó para solução oral - frasco 80 mL</t>
+          <t>0,75 mg/mL pó para solução oral – frasco 80 mL</t>
         </is>
       </c>
     </row>
@@ -13856,7 +13856,7 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>0 - comprimido|5 mg - comprimido</t>
+          <t>0,5 mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -13968,7 +13968,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>0 - comprimido|5mg - comprimido</t>
+          <t>0,5mg – comprimido</t>
         </is>
       </c>
     </row>
@@ -14024,7 +14024,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>50 mcg/g (0 - bisnaga de 30g|005%) pomada - bisnaga de 30g</t>
+          <t>50 mcg/g (0,005%) pomada – bisnaga de 30g</t>
         </is>
       </c>
     </row>
@@ -14192,7 +14192,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>0 - cápsula|25 mcg - cápsula</t>
+          <t>0,25 mcg – cápsula</t>
         </is>
       </c>
     </row>
@@ -14248,7 +14248,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>0 - cápsula|25 mcg - cápsula</t>
+          <t>0,25 mcg – cápsula</t>
         </is>
       </c>
     </row>
@@ -14304,7 +14304,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>0 - cápsula|25 mcg - cápsula</t>
+          <t>0,25 mcg – cápsula</t>
         </is>
       </c>
     </row>
@@ -17448,7 +17448,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>5 - ampola de 1 mL|0 mcg/mL - ampola de 1 mL</t>
+          <t>5,0 mcg/mL – ampola de 1 mL</t>
         </is>
       </c>
     </row>

</xml_diff>